<commit_message>
ci: integrate real E2E tests, security scan, and load testing into unified reports workflow
</commit_message>
<xml_diff>
--- a/tests-e2e/cybershield_test_analysis.xlsx
+++ b/tests-e2e/cybershield_test_analysis.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20 17:42:08</t>
+          <t>2026-07-24 00:32:22</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="F2" s="9" t="n">
-        <v>0.0004834999854210764</v>
+        <v>0.0004292000012355857</v>
       </c>
       <c r="G2" s="8" t="inlineStr"/>
     </row>
@@ -1176,7 +1176,7 @@
         </is>
       </c>
       <c r="F3" s="11" t="n">
-        <v>0.000295900012133643</v>
+        <v>0.0006232999949133955</v>
       </c>
       <c r="G3" s="10" t="inlineStr"/>
     </row>
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>0.0003167999966535717</v>
+        <v>0.0007581000027130358</v>
       </c>
       <c r="G4" s="8" t="inlineStr"/>
     </row>
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="F5" s="11" t="n">
-        <v>0.0002577999839559197</v>
+        <v>0.0007107999990694225</v>
       </c>
       <c r="G5" s="10" t="inlineStr"/>
     </row>
@@ -1269,7 +1269,7 @@
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.0002742999931797385</v>
+        <v>0.0004977999997208826</v>
       </c>
       <c r="G6" s="8" t="inlineStr"/>
     </row>
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.0004978999786544591</v>
+        <v>0.0004139000011491589</v>
       </c>
       <c r="G7" s="10" t="inlineStr"/>
     </row>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.0003089999954681844</v>
+        <v>0.0005750999989686534</v>
       </c>
       <c r="G8" s="8" t="inlineStr"/>
     </row>
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.0002815999905578792</v>
+        <v>0.0004830000034417026</v>
       </c>
       <c r="G9" s="10" t="inlineStr"/>
     </row>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.0003547999949660152</v>
+        <v>0.0004514000029303133</v>
       </c>
       <c r="G10" s="8" t="inlineStr"/>
     </row>
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="F11" s="11" t="n">
-        <v>0.0002886999864131212</v>
+        <v>0.0004631000047083944</v>
       </c>
       <c r="G11" s="10" t="inlineStr"/>
     </row>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0.0002894999925047159</v>
+        <v>0.0005878000010852702</v>
       </c>
       <c r="G12" s="8" t="inlineStr"/>
     </row>
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="F13" s="11" t="n">
-        <v>0.0002514999941922724</v>
+        <v>0.0004179999959887937</v>
       </c>
       <c r="G13" s="10" t="inlineStr"/>
     </row>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="F14" s="9" t="n">
-        <v>0.0003208999987691641</v>
+        <v>0.0003030000007129274</v>
       </c>
       <c r="G14" s="8" t="inlineStr"/>
     </row>
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="F15" s="11" t="n">
-        <v>0.0002684000064618886</v>
+        <v>0.0005000000019208528</v>
       </c>
       <c r="G15" s="10" t="inlineStr"/>
     </row>
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.0002837000065483153</v>
+        <v>0.0004026999959023669</v>
       </c>
       <c r="G16" s="8" t="inlineStr"/>
     </row>
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="F17" s="11" t="n">
-        <v>0.0004720000142697245</v>
+        <v>0.0008165999970515259</v>
       </c>
       <c r="G17" s="10" t="inlineStr"/>
     </row>
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0.0003068000078201294</v>
+        <v>0.0003974999999627471</v>
       </c>
       <c r="G18" s="8" t="inlineStr"/>
     </row>
@@ -1672,7 +1672,7 @@
         </is>
       </c>
       <c r="F19" s="11" t="n">
-        <v>0.0002517000248190016</v>
+        <v>0.0005909000028623268</v>
       </c>
       <c r="G19" s="10" t="inlineStr"/>
     </row>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.0002434999914839864</v>
+        <v>0.0004518999994616024</v>
       </c>
       <c r="G20" s="8" t="inlineStr"/>
     </row>
@@ -1734,7 +1734,7 @@
         </is>
       </c>
       <c r="F21" s="11" t="n">
-        <v>0.0003437999985180795</v>
+        <v>0.0004239999980200082</v>
       </c>
       <c r="G21" s="10" t="inlineStr"/>
     </row>
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="F22" s="9" t="n">
-        <v>0.0004505000251810998</v>
+        <v>0.0004817000008188188</v>
       </c>
       <c r="G22" s="8" t="inlineStr"/>
     </row>
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="F23" s="11" t="n">
-        <v>0.0002731999848037958</v>
+        <v>0.0004217000023345463</v>
       </c>
       <c r="G23" s="10" t="inlineStr"/>
     </row>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.0002519999979995191</v>
+        <v>0.0004404999999678694</v>
       </c>
       <c r="G24" s="8" t="inlineStr"/>
     </row>
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="F25" s="11" t="n">
-        <v>0.0004000999906565994</v>
+        <v>0.0004816999935428612</v>
       </c>
       <c r="G25" s="10" t="inlineStr"/>
     </row>
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="F26" s="9" t="n">
-        <v>0.0003763999848160893</v>
+        <v>0.0006015999970259145</v>
       </c>
       <c r="G26" s="8" t="inlineStr"/>
     </row>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
       <c r="F27" s="11" t="n">
-        <v>0.0005444999842438847</v>
+        <v>0.0004797000001417473</v>
       </c>
       <c r="G27" s="10" t="inlineStr"/>
     </row>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="F28" s="9" t="n">
-        <v>0.0002626000205054879</v>
+        <v>0.0005209000009926967</v>
       </c>
       <c r="G28" s="8" t="inlineStr"/>
     </row>
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="F29" s="11" t="n">
-        <v>0.0006498000002466142</v>
+        <v>0.000371000001905486</v>
       </c>
       <c r="G29" s="10" t="inlineStr"/>
     </row>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="F30" s="9" t="n">
-        <v>0.0004481000069063157</v>
+        <v>0.0003299000018159859</v>
       </c>
       <c r="G30" s="8" t="inlineStr"/>
     </row>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="F31" s="11" t="n">
-        <v>0.0006148999964352697</v>
+        <v>0.0004098999997950159</v>
       </c>
       <c r="G31" s="10" t="inlineStr"/>
     </row>
@@ -2075,7 +2075,7 @@
         </is>
       </c>
       <c r="F32" s="9" t="n">
-        <v>0.0004668000037781894</v>
+        <v>0.0006426000036299229</v>
       </c>
       <c r="G32" s="8" t="inlineStr"/>
     </row>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
       <c r="F33" s="11" t="n">
-        <v>0.0002753000007942319</v>
+        <v>0.0004938999991281889</v>
       </c>
       <c r="G33" s="10" t="inlineStr"/>
     </row>
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="F34" s="9" t="n">
-        <v>0.0003115999861620367</v>
+        <v>0.0003593000001274049</v>
       </c>
       <c r="G34" s="8" t="inlineStr"/>
     </row>
@@ -2168,7 +2168,7 @@
         </is>
       </c>
       <c r="F35" s="11" t="n">
-        <v>0.0006452999950852245</v>
+        <v>0.0006474999972851947</v>
       </c>
       <c r="G35" s="10" t="inlineStr"/>
     </row>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="F36" s="9" t="n">
-        <v>0.0002690000110305846</v>
+        <v>0.0002463999990141019</v>
       </c>
       <c r="G36" s="8" t="inlineStr"/>
     </row>
@@ -2230,7 +2230,7 @@
         </is>
       </c>
       <c r="F37" s="11" t="n">
-        <v>0.0003050999948754907</v>
+        <v>0.0002384000035817735</v>
       </c>
       <c r="G37" s="10" t="inlineStr"/>
     </row>
@@ -2261,7 +2261,7 @@
         </is>
       </c>
       <c r="F38" s="9" t="n">
-        <v>0.0002614000113680959</v>
+        <v>0.0005317000031936914</v>
       </c>
       <c r="G38" s="8" t="inlineStr"/>
     </row>
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="F39" s="11" t="n">
-        <v>0.000395099981687963</v>
+        <v>0.0002268000025651418</v>
       </c>
       <c r="G39" s="10" t="inlineStr"/>
     </row>
@@ -2323,7 +2323,7 @@
         </is>
       </c>
       <c r="F40" s="9" t="n">
-        <v>0.000299600011203438</v>
+        <v>0.0002615000048535876</v>
       </c>
       <c r="G40" s="8" t="inlineStr"/>
     </row>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="F41" s="11" t="n">
-        <v>0.000301799998851493</v>
+        <v>0.0002620000013848767</v>
       </c>
       <c r="G41" s="10" t="inlineStr"/>
     </row>
@@ -2385,7 +2385,7 @@
         </is>
       </c>
       <c r="F42" s="9" t="n">
-        <v>0.000526699994225055</v>
+        <v>0.000458700000308454</v>
       </c>
       <c r="G42" s="8" t="inlineStr"/>
     </row>
@@ -2416,7 +2416,7 @@
         </is>
       </c>
       <c r="F43" s="11" t="n">
-        <v>0.0003351999912410975</v>
+        <v>0.0003550999972503632</v>
       </c>
       <c r="G43" s="10" t="inlineStr"/>
     </row>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="F44" s="9" t="n">
-        <v>0.0002714000002015382</v>
+        <v>0.0005154999962542206</v>
       </c>
       <c r="G44" s="8" t="inlineStr"/>
     </row>
@@ -2478,7 +2478,7 @@
         </is>
       </c>
       <c r="F45" s="11" t="n">
-        <v>0.0002998999843839556</v>
+        <v>0.0004303000023355708</v>
       </c>
       <c r="G45" s="10" t="inlineStr"/>
     </row>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="F46" s="9" t="n">
-        <v>0.0002673999988473952</v>
+        <v>0.0003590999986045063</v>
       </c>
       <c r="G46" s="8" t="inlineStr"/>
     </row>
@@ -2540,7 +2540,7 @@
         </is>
       </c>
       <c r="F47" s="11" t="n">
-        <v>0.0003124999930150807</v>
+        <v>0.0003410999997868203</v>
       </c>
       <c r="G47" s="10" t="inlineStr"/>
     </row>
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="F48" s="9" t="n">
-        <v>0.0002933999930974096</v>
+        <v>0.0002139999996870756</v>
       </c>
       <c r="G48" s="8" t="inlineStr"/>
     </row>
@@ -2602,7 +2602,7 @@
         </is>
       </c>
       <c r="F49" s="11" t="n">
-        <v>0.0004833000130020082</v>
+        <v>0.0004295999970054254</v>
       </c>
       <c r="G49" s="10" t="inlineStr"/>
     </row>
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="F50" s="9" t="n">
-        <v>0.0003180000057909638</v>
+        <v>0.0002652999974088743</v>
       </c>
       <c r="G50" s="8" t="inlineStr"/>
     </row>
@@ -2664,7 +2664,7 @@
         </is>
       </c>
       <c r="F51" s="11" t="n">
-        <v>0.0002697999880183488</v>
+        <v>0.0002811999947880395</v>
       </c>
       <c r="G51" s="10" t="inlineStr"/>
     </row>
@@ -2695,7 +2695,7 @@
         </is>
       </c>
       <c r="F52" s="9" t="n">
-        <v>0.000290700001642108</v>
+        <v>0.0002164000034099445</v>
       </c>
       <c r="G52" s="8" t="inlineStr"/>
     </row>
@@ -2726,7 +2726,7 @@
         </is>
       </c>
       <c r="F53" s="11" t="n">
-        <v>0.0005333000153768808</v>
+        <v>0.000360700003511738</v>
       </c>
       <c r="G53" s="10" t="inlineStr"/>
     </row>
@@ -2757,7 +2757,7 @@
         </is>
       </c>
       <c r="F54" s="9" t="n">
-        <v>0.0002708999963942915</v>
+        <v>0.0002568999989307486</v>
       </c>
       <c r="G54" s="8" t="inlineStr"/>
     </row>
@@ -2788,7 +2788,7 @@
         </is>
       </c>
       <c r="F55" s="11" t="n">
-        <v>0.0002630000235512853</v>
+        <v>0.0004472000000532717</v>
       </c>
       <c r="G55" s="10" t="inlineStr"/>
     </row>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="F56" s="9" t="n">
-        <v>0.0006541000038851053</v>
+        <v>0.0005944000004092231</v>
       </c>
       <c r="G56" s="8" t="inlineStr"/>
     </row>
@@ -2850,7 +2850,7 @@
         </is>
       </c>
       <c r="F57" s="11" t="n">
-        <v>0.0002952999784611166</v>
+        <v>0.0005775000026915222</v>
       </c>
       <c r="G57" s="10" t="inlineStr"/>
     </row>
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="F58" s="9" t="n">
-        <v>0.0002731999848037958</v>
+        <v>0.0006561999980476685</v>
       </c>
       <c r="G58" s="8" t="inlineStr"/>
     </row>
@@ -2912,7 +2912,7 @@
         </is>
       </c>
       <c r="F59" s="11" t="n">
-        <v>0.0002720000047702342</v>
+        <v>0.0008603000023867935</v>
       </c>
       <c r="G59" s="10" t="inlineStr"/>
     </row>
@@ -2943,7 +2943,7 @@
         </is>
       </c>
       <c r="F60" s="9" t="n">
-        <v>0.0003471000236459076</v>
+        <v>0.0006082999971113168</v>
       </c>
       <c r="G60" s="8" t="inlineStr"/>
     </row>
@@ -2974,7 +2974,7 @@
         </is>
       </c>
       <c r="F61" s="11" t="n">
-        <v>0.0004665000014938414</v>
+        <v>0.001203100000566337</v>
       </c>
       <c r="G61" s="10" t="inlineStr"/>
     </row>
@@ -3005,7 +3005,7 @@
         </is>
       </c>
       <c r="F62" s="9" t="n">
-        <v>0.0003117999876849353</v>
+        <v>0.001162599997769576</v>
       </c>
       <c r="G62" s="8" t="inlineStr"/>
     </row>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
       <c r="F63" s="11" t="n">
-        <v>0.0004455999878700823</v>
+        <v>0.0004807000004802831</v>
       </c>
       <c r="G63" s="10" t="inlineStr"/>
     </row>
@@ -3067,7 +3067,7 @@
         </is>
       </c>
       <c r="F64" s="9" t="n">
-        <v>0.0002611000090837479</v>
+        <v>0.0005480999971041456</v>
       </c>
       <c r="G64" s="8" t="inlineStr"/>
     </row>
@@ -3098,7 +3098,7 @@
         </is>
       </c>
       <c r="F65" s="11" t="n">
-        <v>0.0002669999958015978</v>
+        <v>0.0005997999978717417</v>
       </c>
       <c r="G65" s="10" t="inlineStr"/>
     </row>
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="F66" s="9" t="n">
-        <v>0.0002605999761726707</v>
+        <v>0.0005464999994728714</v>
       </c>
       <c r="G66" s="8" t="inlineStr"/>
     </row>
@@ -3160,7 +3160,7 @@
         </is>
       </c>
       <c r="F67" s="11" t="n">
-        <v>0.0004740000003948808</v>
+        <v>0.0005651000028592534</v>
       </c>
       <c r="G67" s="10" t="inlineStr"/>
     </row>
@@ -3191,7 +3191,7 @@
         </is>
       </c>
       <c r="F68" s="9" t="n">
-        <v>0.0002593999961391091</v>
+        <v>0.0005197999998927116</v>
       </c>
       <c r="G68" s="8" t="inlineStr"/>
     </row>
@@ -3222,7 +3222,7 @@
         </is>
       </c>
       <c r="F69" s="11" t="n">
-        <v>0.0002702999918255955</v>
+        <v>0.000691700006427709</v>
       </c>
       <c r="G69" s="10" t="inlineStr"/>
     </row>
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="F70" s="9" t="n">
-        <v>0.0003724999842233956</v>
+        <v>0.00052299999515526</v>
       </c>
       <c r="G70" s="8" t="inlineStr"/>
     </row>
@@ -3284,7 +3284,7 @@
         </is>
       </c>
       <c r="F71" s="11" t="n">
-        <v>0.0003831000067293644</v>
+        <v>0.001016999995044898</v>
       </c>
       <c r="G71" s="10" t="inlineStr"/>
     </row>
@@ -3315,7 +3315,7 @@
         </is>
       </c>
       <c r="F72" s="9" t="n">
-        <v>0.0002589999930933118</v>
+        <v>0.0006591999990632758</v>
       </c>
       <c r="G72" s="8" t="inlineStr"/>
     </row>
@@ -3346,7 +3346,7 @@
         </is>
       </c>
       <c r="F73" s="11" t="n">
-        <v>0.0002835999766830355</v>
+        <v>0.001424399997631554</v>
       </c>
       <c r="G73" s="10" t="inlineStr"/>
     </row>
@@ -3377,7 +3377,7 @@
         </is>
       </c>
       <c r="F74" s="9" t="n">
-        <v>0.0005665000062435865</v>
+        <v>0.0005543000006582588</v>
       </c>
       <c r="G74" s="8" t="inlineStr"/>
     </row>
@@ -3408,7 +3408,7 @@
         </is>
       </c>
       <c r="F75" s="11" t="n">
-        <v>0.0004800999886356294</v>
+        <v>0.0006040000007487833</v>
       </c>
       <c r="G75" s="10" t="inlineStr"/>
     </row>
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="F76" s="9" t="n">
-        <v>0.0004893000004813075</v>
+        <v>0.0005596999981207773</v>
       </c>
       <c r="G76" s="8" t="inlineStr"/>
     </row>
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="F77" s="11" t="n">
-        <v>0.0004538999928627163</v>
+        <v>0.0005414999977801926</v>
       </c>
       <c r="G77" s="10" t="inlineStr"/>
     </row>
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="F78" s="9" t="n">
-        <v>0.0004212999774608761</v>
+        <v>0.0006997999953455292</v>
       </c>
       <c r="G78" s="8" t="inlineStr"/>
     </row>
@@ -3532,7 +3532,7 @@
         </is>
       </c>
       <c r="F79" s="11" t="n">
-        <v>0.0004316999984439462</v>
+        <v>0.001078100001905113</v>
       </c>
       <c r="G79" s="10" t="inlineStr"/>
     </row>
@@ -3563,7 +3563,7 @@
         </is>
       </c>
       <c r="F80" s="9" t="n">
-        <v>0.000311399984639138</v>
+        <v>0.0007432999991578981</v>
       </c>
       <c r="G80" s="8" t="inlineStr"/>
     </row>
@@ -3594,7 +3594,7 @@
         </is>
       </c>
       <c r="F81" s="11" t="n">
-        <v>0.0003176000027451664</v>
+        <v>0.0007279999990714714</v>
       </c>
       <c r="G81" s="10" t="inlineStr"/>
     </row>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="F82" s="9" t="n">
-        <v>0.0006533999985549599</v>
+        <v>0.0006884000031277537</v>
       </c>
       <c r="G82" s="8" t="inlineStr"/>
     </row>
@@ -3656,7 +3656,7 @@
         </is>
       </c>
       <c r="F83" s="11" t="n">
-        <v>0.0003342999843880534</v>
+        <v>0.0006403000006685033</v>
       </c>
       <c r="G83" s="10" t="inlineStr"/>
     </row>
@@ -3687,7 +3687,7 @@
         </is>
       </c>
       <c r="F84" s="9" t="n">
-        <v>0.0003788999747484922</v>
+        <v>0.0005479999963426962</v>
       </c>
       <c r="G84" s="8" t="inlineStr"/>
     </row>
@@ -3718,7 +3718,7 @@
         </is>
       </c>
       <c r="F85" s="11" t="n">
-        <v>0.0003075999848078936</v>
+        <v>0.0005596000046352856</v>
       </c>
       <c r="G85" s="10" t="inlineStr"/>
     </row>
@@ -3749,7 +3749,7 @@
         </is>
       </c>
       <c r="F86" s="9" t="n">
-        <v>0.0002893999917432666</v>
+        <v>0.0005144000024301931</v>
       </c>
       <c r="G86" s="8" t="inlineStr"/>
     </row>
@@ -3780,7 +3780,7 @@
         </is>
       </c>
       <c r="F87" s="11" t="n">
-        <v>0.0002707999956328422</v>
+        <v>0.0007047999970382079</v>
       </c>
       <c r="G87" s="10" t="inlineStr"/>
     </row>
@@ -3811,7 +3811,7 @@
         </is>
       </c>
       <c r="F88" s="9" t="n">
-        <v>0.0006968000088818371</v>
+        <v>0.0006993999995756894</v>
       </c>
       <c r="G88" s="8" t="inlineStr"/>
     </row>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="F89" s="11" t="n">
-        <v>0.0003623999946285039</v>
+        <v>0.0004651999988709576</v>
       </c>
       <c r="G89" s="10" t="inlineStr"/>
     </row>
@@ -3873,7 +3873,7 @@
         </is>
       </c>
       <c r="F90" s="9" t="n">
-        <v>0.0003006000188179314</v>
+        <v>0.0005180000007385388</v>
       </c>
       <c r="G90" s="8" t="inlineStr"/>
     </row>
@@ -3904,7 +3904,7 @@
         </is>
       </c>
       <c r="F91" s="11" t="n">
-        <v>0.0003519999736454338</v>
+        <v>0.0004524999967543408</v>
       </c>
       <c r="G91" s="10" t="inlineStr"/>
     </row>
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="F92" s="9" t="n">
-        <v>0.0003488000074867159</v>
+        <v>0.0005183999965083785</v>
       </c>
       <c r="G92" s="8" t="inlineStr"/>
     </row>
@@ -3966,7 +3966,7 @@
         </is>
       </c>
       <c r="F93" s="11" t="n">
-        <v>0.0004182999837212265</v>
+        <v>0.0005703999995603226</v>
       </c>
       <c r="G93" s="10" t="inlineStr"/>
     </row>
@@ -3997,7 +3997,7 @@
         </is>
       </c>
       <c r="F94" s="9" t="n">
-        <v>0.0006095999851822853</v>
+        <v>0.0005848000000696629</v>
       </c>
       <c r="G94" s="8" t="inlineStr"/>
     </row>
@@ -4028,7 +4028,7 @@
         </is>
       </c>
       <c r="F95" s="11" t="n">
-        <v>0.0003365000011399388</v>
+        <v>0.0004157000003033318</v>
       </c>
       <c r="G95" s="10" t="inlineStr"/>
     </row>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="F96" s="9" t="n">
-        <v>0.0003009999927598983</v>
+        <v>0.0006596000021090731</v>
       </c>
       <c r="G96" s="8" t="inlineStr"/>
     </row>
@@ -4090,7 +4090,7 @@
         </is>
       </c>
       <c r="F97" s="11" t="n">
-        <v>0.0002744999947026372</v>
+        <v>0.0005225999993854202</v>
       </c>
       <c r="G97" s="10" t="inlineStr"/>
     </row>
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="F98" s="9" t="n">
-        <v>0.0003164999943692237</v>
+        <v>0.0005480999971041456</v>
       </c>
       <c r="G98" s="8" t="inlineStr"/>
     </row>
@@ -4152,7 +4152,7 @@
         </is>
       </c>
       <c r="F99" s="11" t="n">
-        <v>0.0003258000069763511</v>
+        <v>0.0007165999995777383</v>
       </c>
       <c r="G99" s="10" t="inlineStr"/>
     </row>
@@ -4183,7 +4183,7 @@
         </is>
       </c>
       <c r="F100" s="9" t="n">
-        <v>0.0002948999754153192</v>
+        <v>0.0004186000005574897</v>
       </c>
       <c r="G100" s="8" t="inlineStr"/>
     </row>
@@ -4214,7 +4214,7 @@
         </is>
       </c>
       <c r="F101" s="11" t="n">
-        <v>0.001067899982444942</v>
+        <v>0.001042100004269741</v>
       </c>
       <c r="G101" s="10" t="inlineStr"/>
     </row>
@@ -4245,7 +4245,7 @@
         </is>
       </c>
       <c r="F102" s="9" t="n">
-        <v>0.000377199990907684</v>
+        <v>0.0005120999994687736</v>
       </c>
       <c r="G102" s="8" t="inlineStr"/>
     </row>
@@ -4276,7 +4276,7 @@
         </is>
       </c>
       <c r="F103" s="11" t="n">
-        <v>0.0002914999786298722</v>
+        <v>0.0004925000030198134</v>
       </c>
       <c r="G103" s="10" t="inlineStr"/>
     </row>
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="F104" s="9" t="n">
-        <v>0.0003862000012304634</v>
+        <v>0.0005939000038779341</v>
       </c>
       <c r="G104" s="8" t="inlineStr"/>
     </row>
@@ -4338,7 +4338,7 @@
         </is>
       </c>
       <c r="F105" s="11" t="n">
-        <v>0.0004119999939575791</v>
+        <v>0.0007839999962016009</v>
       </c>
       <c r="G105" s="10" t="inlineStr"/>
     </row>
@@ -4369,7 +4369,7 @@
         </is>
       </c>
       <c r="F106" s="9" t="n">
-        <v>0.001249900000402704</v>
+        <v>0.0006070999952498823</v>
       </c>
       <c r="G106" s="8" t="inlineStr"/>
     </row>
@@ -4400,7 +4400,7 @@
         </is>
       </c>
       <c r="F107" s="11" t="n">
-        <v>0.000374099996406585</v>
+        <v>0.0006946999928914011</v>
       </c>
       <c r="G107" s="10" t="inlineStr"/>
     </row>
@@ -4431,7 +4431,7 @@
         </is>
       </c>
       <c r="F108" s="9" t="n">
-        <v>0.0003307000151835382</v>
+        <v>0.0006357000020216219</v>
       </c>
       <c r="G108" s="8" t="inlineStr"/>
     </row>
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="F109" s="11" t="n">
-        <v>0.0003457999846432358</v>
+        <v>0.0005368999991333112</v>
       </c>
       <c r="G109" s="10" t="inlineStr"/>
     </row>

</xml_diff>